<commit_message>
finish 05; start 06 material
</commit_message>
<xml_diff>
--- a/data/schedule.xlsx
+++ b/data/schedule.xlsx
@@ -786,6 +786,11 @@
       <c r="I7" t="s">
         <v>39</v>
       </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>/assignment/06-assignment-cleaning</t>
+        </is>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">

</xml_diff>